<commit_message>
update Myrans_2021 (final), Ottaviani_2015 (near final)
</commit_message>
<xml_diff>
--- a/data/Myrans_2021/raw/Myrans_2021 raw data.xlsx
+++ b/data/Myrans_2021/raw/Myrans_2021 raw data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PhD\N trial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CE26DC9-5FAD-47F0-B337-BFADB0BE0C07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B32A1F7-F893-4C64-8F6B-31D79D4BDE65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" activeTab="1" xr2:uid="{A837CD8B-1446-4DBA-BEE5-9CD0B5B69848}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" activeTab="5" xr2:uid="{A837CD8B-1446-4DBA-BEE5-9CD0B5B69848}"/>
   </bookViews>
   <sheets>
     <sheet name="S. bicolor" sheetId="1" r:id="rId1"/>
@@ -10392,13 +10392,13 @@
         <v>1.4125207420122278E-2</v>
       </c>
       <c r="Z2">
-        <v>55.752125169397559</v>
+        <v>1.21</v>
       </c>
       <c r="AA2">
-        <v>19.455463841320686</v>
+        <v>0.94</v>
       </c>
       <c r="AB2">
-        <v>24.792410989281759</v>
+        <v>0.78</v>
       </c>
       <c r="AC2">
         <v>70</v>
@@ -10478,13 +10478,13 @@
         <v>1.5024017096244841E-2</v>
       </c>
       <c r="Z3">
-        <v>51.833665366592776</v>
+        <v>0.91</v>
       </c>
       <c r="AA3">
-        <v>21.296893852240515</v>
+        <v>0.69</v>
       </c>
       <c r="AB3">
-        <v>26.869440781166698</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="AC3">
         <v>68</v>
@@ -10567,13 +10567,13 @@
         <v>5.0973048184177689E-3</v>
       </c>
       <c r="Z4">
-        <v>50.532123368205248</v>
+        <v>1.1100000000000001</v>
       </c>
       <c r="AA4">
-        <v>27.109650577346319</v>
+        <v>0.8</v>
       </c>
       <c r="AB4">
-        <v>22.35822605444843</v>
+        <v>0.72</v>
       </c>
       <c r="AC4">
         <v>69</v>
@@ -10647,13 +10647,13 @@
         <v>5.9929206577461237E-3</v>
       </c>
       <c r="Z5">
-        <v>61.935431273438759</v>
+        <v>1.07</v>
       </c>
       <c r="AA5">
-        <v>26.438936898744497</v>
+        <v>0.94</v>
       </c>
       <c r="AB5">
-        <v>11.625631827816727</v>
+        <v>0.62</v>
       </c>
       <c r="AC5">
         <v>69</v>
@@ -10777,13 +10777,13 @@
         <v>3.2997369585726334E-2</v>
       </c>
       <c r="Z7">
-        <v>54.286937214092724</v>
+        <v>0.91</v>
       </c>
       <c r="AA7">
-        <v>20.432840212942409</v>
+        <v>0.67</v>
       </c>
       <c r="AB7">
-        <v>25.280222572964878</v>
+        <v>0.6</v>
       </c>
       <c r="AC7">
         <v>70</v>
@@ -10863,13 +10863,13 @@
         <v>9.1513702233669308E-2</v>
       </c>
       <c r="Z8">
-        <v>32.86373656654726</v>
+        <v>0.94</v>
       </c>
       <c r="AA8">
-        <v>42.925048222650872</v>
+        <v>0.62</v>
       </c>
       <c r="AB8">
-        <v>24.211215210801875</v>
+        <v>0.66</v>
       </c>
       <c r="AC8">
         <v>67</v>
@@ -10949,13 +10949,13 @@
         <v>0.17170888878654078</v>
       </c>
       <c r="Z9">
-        <v>55.581010932923483</v>
+        <v>0.74</v>
       </c>
       <c r="AA9">
-        <v>17.704376069367516</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="AB9">
-        <v>26.714612997709015</v>
+        <v>0.47</v>
       </c>
       <c r="AC9">
         <v>70</v>
@@ -11035,13 +11035,13 @@
         <v>2.3270440237995998E-3</v>
       </c>
       <c r="Z10">
-        <v>52.141849137342376</v>
+        <v>0.83</v>
       </c>
       <c r="AA10">
-        <v>24.254563663677335</v>
+        <v>0.72</v>
       </c>
       <c r="AB10">
-        <v>23.603587198980289</v>
+        <v>0.61</v>
       </c>
       <c r="AC10">
         <v>69</v>
@@ -11121,13 +11121,13 @@
         <v>2.901661085689897E-2</v>
       </c>
       <c r="Z11">
-        <v>54.530130239478666</v>
+        <v>1.85</v>
       </c>
       <c r="AA11">
-        <v>24.129617945361574</v>
+        <v>1.08</v>
       </c>
       <c r="AB11">
-        <v>21.340251815159764</v>
+        <v>0.86</v>
       </c>
       <c r="AC11">
         <v>67</v>
@@ -11204,13 +11204,13 @@
         <v>0.16219227761519314</v>
       </c>
       <c r="Z12">
-        <v>50.526363916924801</v>
+        <v>2.57</v>
       </c>
       <c r="AA12">
-        <v>27.263479145473045</v>
+        <v>1.78</v>
       </c>
       <c r="AB12">
-        <v>22.210156937602161</v>
+        <v>1.27</v>
       </c>
       <c r="AC12">
         <v>74</v>
@@ -11293,13 +11293,13 @@
         <v>4.0665494083110251E-2</v>
       </c>
       <c r="Z13">
-        <v>58.677889169720196</v>
+        <v>1.51</v>
       </c>
       <c r="AA13">
-        <v>24.902347292933932</v>
+        <v>1.17</v>
       </c>
       <c r="AB13">
-        <v>16.419763537345862</v>
+        <v>0.77</v>
       </c>
       <c r="AC13">
         <v>68</v>
@@ -11376,13 +11376,13 @@
         <v>0.2081379082785548</v>
       </c>
       <c r="Z14">
-        <v>53.791521029875121</v>
+        <v>2.09</v>
       </c>
       <c r="AA14">
-        <v>41.251786038415531</v>
+        <v>1.82</v>
       </c>
       <c r="AB14">
-        <v>4.9566929317093376</v>
+        <v>1.42</v>
       </c>
       <c r="AC14">
         <v>70</v>
@@ -11465,13 +11465,13 @@
         <v>0.19563236195880557</v>
       </c>
       <c r="Z15">
-        <v>45.021645021645021</v>
+        <v>1.86</v>
       </c>
       <c r="AA15">
-        <v>24.637420950785007</v>
+        <v>1.5</v>
       </c>
       <c r="AB15">
-        <v>30.340934027569975</v>
+        <v>1.34</v>
       </c>
       <c r="AC15">
         <v>68</v>
@@ -11554,13 +11554,13 @@
         <v>9.5323687408005991E-3</v>
       </c>
       <c r="Z16">
-        <v>55.32508603850804</v>
+        <v>1.44</v>
       </c>
       <c r="AA16">
-        <v>26.970100972519351</v>
+        <v>1.1200000000000001</v>
       </c>
       <c r="AB16">
-        <v>17.704812988972602</v>
+        <v>0.74</v>
       </c>
       <c r="AC16">
         <v>69</v>
@@ -11643,13 +11643,13 @@
         <v>1.3127828467740304E-2</v>
       </c>
       <c r="Z17">
-        <v>57.091023820791918</v>
+        <v>2.31</v>
       </c>
       <c r="AA17">
-        <v>29.804911395067567</v>
+        <v>1.82</v>
       </c>
       <c r="AB17">
-        <v>13.104064784140505</v>
+        <v>0.98</v>
       </c>
       <c r="AC17">
         <v>69</v>
@@ -11732,13 +11732,13 @@
         <v>4.471995967849858E-2</v>
       </c>
       <c r="Z18">
-        <v>59.988845637278331</v>
+        <v>1.66</v>
       </c>
       <c r="AA18">
-        <v>22.425960071934259</v>
+        <v>1.22</v>
       </c>
       <c r="AB18">
-        <v>17.585194290787406</v>
+        <v>0.9</v>
       </c>
       <c r="AC18">
         <v>69</v>

</xml_diff>